<commit_message>
feat: improve information on results.xlsx report
</commit_message>
<xml_diff>
--- a/src/results.xlsx
+++ b/src/results.xlsx
@@ -413,69 +413,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>session_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>act_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>test_case_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>num_steps_executed</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>result</t>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>test_passed</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3f39ee03-77bc-4325-84e6-a567ea224d7a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>9d9b1914-7a4c-40db-b232-7fb4520c0890</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Validar el flujo de inicio de sesión desde el ingreso de credenciales hasta la visualización del mensaje de bienvenida en el header.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>❌ Step failed: No response from agent</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>El usuario hace click en el campo 'Correo electrónico', format output with jsonschema: {"properties": {"test_passed": {"title": "Test Passed", "type": "boolean"}, "error": {"anyOf": [{"type": "string"}, {"type": "null"}], "default": null, "title": "Error"}}, "required": ["test_passed"], "title": "TestResult", "type": "object"}</t>
+        </is>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Validation failed: 1 validation error for TestResult
+  Input should be a valid dictionary or instance of TestResult [type=model_type, input_value=None, input_type=NoneType]
+    For further information visit https://errors.pydantic.dev/2.11/v/model_type</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1c505c20-6e55-4ec4-b6bd-f4f1f3ea5514</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>d37beb9f-f420-4ca6-9e57-f290d54ef4ca</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Verificar que el usuario pueda iniciar correctamente una partida en el juego de memorama y manejar errores si ocurren.</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>❌ Step failed: El botÃ³n Jugar no estÃ¡ visible, se requiere corregir los errores en el formulario.</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>El usuario hace click en el botón Jugar, en caso de error retorna un error</t>
+        </is>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>The 'Jugar' button is not available.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3435a2b1-2885-4581-a2dc-c7032e49fd7d</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>46cba05d-43ab-4f9f-9589-22c14fb3b0ac</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Comprobar que se muestre la escala de tolerancia, permitir la selección de un nivel y mostrar la pregunta asociada al producto.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>✅ All steps passed</t>
-        </is>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Se visualiza el texto ¿Aceptarías este producto en tu vida?, format output with jsonschema: {"properties": {"test_passed": {"title": "Test Passed", "type": "boolean"}, "error": {"anyOf": [{"type": "string"}, {"type": "null"}], "default": null, "title": "Error"}}, "required": ["test_passed"], "title": "TestResult", "type": "object"}</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>